<commit_message>
Leads: 2026-09-20 18:38 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -644,7 +644,6 @@
           <t>https://www.mt406hvac.com/</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>service@mt406hvac.com</t>
@@ -674,6 +673,122 @@
         </is>
       </c>
       <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Emergency Plumber San Jose | 24/7 Fast Response</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>plumbingcontractorsanjoseca.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://plumbingcontractorsanjoseca.com/emergency-plumbing.html</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>How It</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>info@plumbingcontractorsanjoseca.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(408) 403-3102</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>San Jose CA</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>emergency plumber San Jose CA</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>HVAC Contractor | Casper, WY | Cole Custom Air</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>colecustomair.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.colecustomair.com/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>colecustomair@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(307) 265-8926</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Casper WY</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>88</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>HVAC contractor Casper WY</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 18:40 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -759,7 +759,6 @@
           <t>https://www.colecustomair.com/</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>colecustomair@yahoo.com</t>
@@ -789,6 +788,62 @@
         </is>
       </c>
       <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>edgelineroofingservices.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://edgelineroofingservices.com/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>sales@edgelineroofingservices.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(916) 633 6692</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Elk Grove CA</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>80</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>residential roofing company Elk Grove CA</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 18:43 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -814,7 +814,6 @@
           <t>https://edgelineroofingservices.com/</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>sales@edgelineroofingservices.com</t>
@@ -844,6 +843,118 @@
         </is>
       </c>
       <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HVAC &amp; Refrigeration | Salinas, CA | Fairwinds Refrigeration</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>fairwindsrefrigerationandhvac.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://www.fairwindsrefrigerationandhvac.com/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>fairwindsrefrigeration.hvac@gmail.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(844) 777-9060</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Salinas CA</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>80</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>AC installation Salinas CA</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>A &amp; M Metal Roofing Innovations</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ammetalroofing.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://ammetalroofing.com/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>contact@ammetalroofing.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(830) 624-9941</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>80</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>metal roofing contractor New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 18:44 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -869,7 +869,6 @@
           <t>https://www.fairwindsrefrigerationandhvac.com/</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>fairwindsrefrigeration.hvac@gmail.com</t>
@@ -925,7 +924,6 @@
           <t>https://ammetalroofing.com/</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>contact@ammetalroofing.com</t>
@@ -955,6 +953,66 @@
         </is>
       </c>
       <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>draincleaningnaperville.com</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>draincleaningnaperville.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://draincleaningnaperville.com/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Why Choose</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>info@draincleaningnaperville.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(331)315-0300</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Naperville IL</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>98</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>drain cleaning service Naperville IL</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 18:47 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1018,6 +1018,62 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>lc-plumbingandgas.com</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>lc-plumbingandgas.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.lc-plumbingandgas.com/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>lcplumbingandgas@gmail.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(575) 223-2580</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Las Cruces NM</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>68</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>plumbing company Las Cruces NM</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 18:57 UTC (cycle 16)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1039,7 +1039,6 @@
           <t>https://www.lc-plumbingandgas.com/</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>lcplumbingandgas@gmail.com</t>
@@ -1069,6 +1068,118 @@
         </is>
       </c>
       <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Integrity Roofing &amp; Restoration LLC</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>integrityroofingofnc.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://www.integrityroofingofnc.com/fayetteville-nc/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>integrityroofingllc2@gmail.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(919) 327-0553</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Fayetteville NC</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>98</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>residential roofing company Fayetteville NC</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Advanced Roofing Solutions, LLC. |</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>advancedroofingsolutionsllc.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://advancedroofingsolutionsllc.com/residential-roofing-fayetteville-nc/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>teamtonet@gmail.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(910) 988-8245</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Fayetteville NC</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>98</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>residential roofing company Fayetteville NC</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 18:59 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1094,7 +1094,6 @@
           <t>https://www.integrityroofingofnc.com/fayetteville-nc/</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>integrityroofingllc2@gmail.com</t>
@@ -1150,7 +1149,6 @@
           <t>https://advancedroofingsolutionsllc.com/residential-roofing-fayetteville-nc/</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>teamtonet@gmail.com</t>
@@ -1180,6 +1178,66 @@
         </is>
       </c>
       <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>AXIS Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>axisairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://axisairconditioning.com/areas/tempe-az</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>How We</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>blake@axisairconditioning.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(480) 571-1515</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Tempe AZ</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>98</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>HVAC contractor Tempe AZ</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 19:06 UTC (cycle 22)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1243,6 +1243,62 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>HVAC Contractor | Air Quality Mechanical</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>airqualitymechanical.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.airqualitymechanical.com/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>info@airqualitymechanical.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(406) 721-7018</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Missoula MT</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>HVAC contractor Missoula MT</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 19:08 UTC (cycle 23)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1264,7 +1264,6 @@
           <t>https://www.airqualitymechanical.com/</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>info@airqualitymechanical.com</t>
@@ -1294,6 +1293,66 @@
         </is>
       </c>
       <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Zion Custom Air Inc</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>zioncustomair.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://www.zioncustomair.com/heat-pumps-installation-repair-palmdale-ca.php</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Santa Clarita</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>info@zioncustomair.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>661-361-3535</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Palmdale CA</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>90</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>heat pump installation Palmdale CA</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 19:18 UTC (cycle 30)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1358,6 +1358,66 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Expertise Plumbing &amp; Rooter</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>expertiseplumbing.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://expertiseplumbing.com/plumbing-services/emergency-plumber-los-angeles/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Who We</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>info@expertiseplumbing.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>888-807-7069</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>100</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>emergency plumber Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 19:19 UTC (cycle 31)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1418,6 +1418,126 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>The Bethlehem Plumber</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>thebethlehemplumber.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://thebethlehemplumber.com/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Catasauqua Rd</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>info@thebethlehemplumber.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>(610) 885 4760</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>100</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>emergency plumber Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Young Plumbing</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>youngplumbingllc.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.youngplumbingllc.com/emergency-plumbing-services</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Joshua Young</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>youngplumbingllc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>610-867-5682</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>90</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>emergency plumber Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 19:21 UTC (cycle 32)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1538,6 +1538,126 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Macklen Home Builders and Roofing</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>macklenroofing.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://macklenroofing.com/</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Macklen Home</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>macklenhbr@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>843-430-3548</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Myrtle Beach SC</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>100</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>roof repair company Myrtle Beach SC</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Golden Roofing</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>goldenroofingsc.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://goldenroofingsc.com/</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Homeowner Guides</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>goldenroofingmb@gmail.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>(843) 655-2402</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Myrtle Beach SC</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>90</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>roof repair company Myrtle Beach SC</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 19:25 UTC (cycle 35)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1658,6 +1658,182 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Big Dog Roofing</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>bigdogroofing.org</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://www.bigdogroofing.org/services/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Member Matt</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>team@bigdogroofing.org</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>260.999.0347</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>90</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Weavers Roofing &amp; Construction, LLC</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>metalrooffortwaynein.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>http://metalrooffortwaynein.com/</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>moreinfo@metalrooffortwaynein.com</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>260-202-4456</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>84</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Emergency Plumber in Chandler, AZ | Chandler Plumbing Co.</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>plumbingchandlerarizona.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>http://plumbingchandlerarizona.com/</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Sun Lakes</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>info@plumbingchandlerarizona.com</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>(607) 302-4614</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Chandler AZ</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>78</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>sewer repair Chandler AZ</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 19:28 UTC (cycle 37)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1739,7 +1739,6 @@
           <t>http://metalrooffortwaynein.com/</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>moreinfo@metalrooffortwaynein.com</t>
@@ -1829,6 +1828,66 @@
         </is>
       </c>
       <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Hydro Jet Drain Service</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>hydrojetdrainservice.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://hydrojetdrainservice.com/services/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Toms River</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>hydrojetdrainservice@gmail.com</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>(732) 523 5217</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Toms River NJ</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>94</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>drain cleaning service Toms River NJ</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 19:33 UTC (cycle 40)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1893,6 +1893,62 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Bellingham Plumbers</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>favingerplumbing.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://www.favingerplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>info@favingerplumbing.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>360-676-1774</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Bellingham WA</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>100</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>plumber Bellingham WA</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 19:34 UTC (cycle 41)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1914,7 +1914,6 @@
           <t>https://www.favingerplumbing.com/</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>info@favingerplumbing.com</t>
@@ -1944,6 +1943,66 @@
         </is>
       </c>
       <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Fox Plumbing &amp; Heating Services</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>foxplumbingak.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://foxplumbingak.com/</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Heating Your</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>foxplumbing49@gmail.com</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>(907) 830-3499</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Anchorage AK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>90</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>plumber Anchorage AK</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 19:38 UTC (cycle 44)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2008,6 +2008,58 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>cavalleroheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>http://cavalleroheatingandair.com/</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>info@cavalleroheatingandair.com</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>(775) 883-2066</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Carson City NV</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>48</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>HVAC contractor Carson City NV</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 19:44 UTC (cycle 48)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2009,7 +2009,6 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
           <t>HVAC</t>
@@ -2025,7 +2024,6 @@
           <t>http://cavalleroheatingandair.com/</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>info@cavalleroheatingandair.com</t>
@@ -2055,6 +2053,66 @@
         </is>
       </c>
       <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Roofing Contractor Memphis TN | Home Restoration</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>homerestorationmemphis.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://www.homerestorationmemphis.com/</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Home Restoration</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>homerestorations37@gmail.com</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>(901) 406-1720</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Memphis TN</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>100</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>roofing contractor Memphis TN</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 19:47 UTC (cycle 50)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2118,6 +2118,66 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>CCC Roofing and Construction</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>cccroofingandconstruction.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://cccroofingandconstruction.com/</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Client Testimonials</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>jakec200@gmail.com</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>(405) 473-2942</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Edmond OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>100</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>roofing contractor Edmond OK</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 19:54 UTC (cycle 55)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2178,6 +2178,66 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>HVAC Company | Cold Front A/C of The Woodlands | The Woodlands &amp; Conroe, TX</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>coldfrontacofthewoodlands.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://www.coldfrontacofthewoodlands.com/</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>At Cold</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>coldfrontacofthewoodlands@gmail.com</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>832-559-8236</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>The Woodlands TX</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>90</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>HVAC contractor The Woodlands TX</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 20:06 UTC (cycle 63)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2238,6 +2238,66 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Precise Air &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>preciseairandheating.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://preciseairandheating.com/ac-repair-mesa-az</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Encanto Call</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>eben@eyebytes.com</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>(602) 396-0869</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Mesa AZ</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>90</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>air conditioning repair Mesa AZ</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 20:10 UTC (cycle 66)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2298,6 +2298,66 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Otterwise Plumbing</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>otterwiseservices.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://otterwiseservices.com/plumbing-services/sewer-and-drain-services/sewer-line-repair-replacement/</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Carter Lovinggood</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>otterwiseplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>(801) 837-6622</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Ogden UT</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>90</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>sewer repair Ogden UT</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 20:22 UTC (cycle 74)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2358,6 +2358,66 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Roofing Contractor Baton Rouge LA</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>pgroofingandconstruction.co</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://pgroofingandconstruction.co/</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Preaux Geaux</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>roy@pgroofingandconstruction.co</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>225-252-5262</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Baton Rouge LA</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>76</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>roofing contractor Baton Rouge LA</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 20:48 UTC (cycle 92)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2418,6 +2418,66 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Big Timber Roofing</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>bigtimberroofing.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://bigtimberroofing.com/</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Get Free</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>bigtimberroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>931-472-5055</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Clarksville TN</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>76</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>roofer Clarksville TN</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 20:49 UTC (cycle 93)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2478,6 +2478,66 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Plumbing in Stockton, CA | JVS Plumbing</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>jvsplumb.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://www.jvsplumb.com/emergency-plumber-stockton-ca</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Homeowners Property</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>jvsplumbing1@gmail.com</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>(209) 229-5487</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Stockton CA</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>90</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>emergency plumber Stockton CA</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 20:54 UTC (cycle 96)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2538,6 +2538,126 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>RD Plumbing and Rooter</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>rdplumbingrooter.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://rdplumbingrooter.com/</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Claudia Elena</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>rdplumbingandrooterinfo@gmail.com</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>951-800-3320</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Riverside CA</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>90</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>emergency plumber Riverside CA</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Evergreen Plumbing Riverside</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>evergreenplumbingriverside.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://evergreenplumbingriverside.com/24-7-emergency-plumbing-services/</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Why Riverside</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>info@evergreenplumbingriverside.com</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>(951) 309-5599</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Riverside CA</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>80</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>emergency plumber Riverside CA</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 20:58 UTC (cycle 99)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2658,6 +2658,122 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Roofing in Anchorage, AK | Twin Point Roofing</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>twinpointroofing-ak.com</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://twinpointroofing-ak.com/services/roofing-replacement/</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Roofing Replacement</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>twinpointroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>(907) 615-1772</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Anchorage AK</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>96</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>roof replacement Anchorage AK</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>AC installation in San Marcos</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>austinhvacsolutions.com</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://austinhvacsolutions.com/locations/san-marcos-tx/ac-installation</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>info@austinhvacsolutions.com</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>(512) 877-2104</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>San Marcos TX</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>90</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>AC installation San Marcos TX</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 21:14 UTC (cycle 110)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2739,7 +2739,6 @@
           <t>https://austinhvacsolutions.com/locations/san-marcos-tx/ac-installation</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>info@austinhvacsolutions.com</t>
@@ -2769,6 +2768,66 @@
         </is>
       </c>
       <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>The Roofing &amp; Siding Company</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>roofingandsiding.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://www.roofingandsiding.com/service-areas/thornton</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Free Roof</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>hello@roofingandsiding.com</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>303.351.1561</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Thornton CO</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>100</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>roofing contractor Thornton CO</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 21:25 UTC (cycle 118)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2833,6 +2833,66 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>TSC Air</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>tscair.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://tscair.com/</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Owners Don</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>info@tscair.com</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>480 460 1487</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Tempe AZ</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>88</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>furnace repair Tempe AZ</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 21:33 UTC (cycle 123)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2893,6 +2893,66 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Kyle Plumbing</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>kyleplumbing.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://www.kyleplumbing.com/pompano-beach/</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>South Florida</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>service@kyleplumbing.com</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>(754) 256-3630</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Pompano Beach FL</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>100</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>plumbing company Pompano Beach FL</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 21:35 UTC (cycle 125)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2953,6 +2953,66 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Berico</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>berico.com</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://www.berico.com/</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Will Berry</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>inforequest@berico.com</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>336-273-8663</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Greensboro NC</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>100</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>furnace repair Greensboro NC</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 21:38 UTC (cycle 127)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3013,6 +3013,66 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>HVAC Contractor - Lexington, KY</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>stewartac.com</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://www.stewartac.com/</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Services Heating</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>j@stewartac.com</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>859-252-4945</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Lexington KY</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>90</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>HVAC contractor Lexington KY</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 21:41 UTC (cycle 129)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3073,6 +3073,66 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Roofing Contractor in Columbia, MO | Chavez Enterprises</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>thechavezenterprises.com</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://www.thechavezenterprises.com/roofing-columbia-mo</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Chavez Enterprises</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>office@thechavezenterprises.com</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>(573) 821-7663</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Columbia MO</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>90</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>roofing contractor Columbia MO</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 21:44 UTC (cycle 131)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3133,6 +3133,66 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>BestPros Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>bestprosheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://bestprosheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Nathan Anderson</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>info@bestprosheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>(720) 712-7314</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Lakewood CO</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>90</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>HVAC contractor Lakewood CO</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 21:46 UTC (cycle 132)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3193,6 +3193,62 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Plumber in Irvine, CA 24/7 ⭐⭐⭐⭐⭐ - Free Estimate</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>plumberinirvine247.com</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>http://www.plumberinirvine247.com/</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>admin@plumberinirvine247.com</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>(949) 531-7058</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Irvine CA</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>78</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>emergency plumber Irvine CA</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 21:52 UTC (cycle 136)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3214,7 +3214,6 @@
           <t>http://www.plumberinirvine247.com/</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
           <t>admin@plumberinirvine247.com</t>
@@ -3244,6 +3243,66 @@
         </is>
       </c>
       <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>G.R.M Roofing</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>grm-roofing.com</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://www.grm-roofing.com/roofing-toms-river-nj</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Little Egg</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>chasemartin@grm-roofing.com</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>(609) 389-2485</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Toms River NJ</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>90</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>roofing contractor Toms River NJ</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 21:54 UTC (cycle 138)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3308,6 +3308,62 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Air Houston Mechanical</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>airhoustonmechanical.com</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://www.airhoustonmechanical.com/furnaces/furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>info@airhoustonacservices.com</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>832-780-3765</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Conroe TX</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>100</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>furnace repair Conroe TX</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 21:56 UTC (cycle 139)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3329,7 +3329,6 @@
           <t>https://www.airhoustonmechanical.com/furnaces/furnace-repair/</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
           <t>info@airhoustonacservices.com</t>
@@ -3359,6 +3358,66 @@
         </is>
       </c>
       <c r="L50" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Kasidonis Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>kasidonisheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://kasidonisheatingandcooling.com/services/heat-pump-installation</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Blog Privacy</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>service@kasidonisheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>(330) 870-9492</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Columbus OH</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>90</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>heat pump installation Columbus OH</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 21:59 UTC (cycle 141)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3423,6 +3423,62 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Sewer Repair | Los Angeles, CA | Top Contender Drain Specialist</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>topcontenderds.com</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://www.topcontenderds.com/sewer-repair/los-angeles-ca</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>topcontender09@aol.com</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>818-581-8993</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>100</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>sewer repair Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 22:00 UTC (cycle 142)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3444,7 +3444,6 @@
           <t>https://www.topcontenderds.com/sewer-repair/los-angeles-ca</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
           <t>topcontender09@aol.com</t>
@@ -3474,6 +3473,62 @@
         </is>
       </c>
       <c r="L52" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Frog Heating, Air &amp; Electrical</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>frogair.com</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://frogair.com/</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>wecare@frogair.com</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>615.657.4351</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Nashville TN</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>90</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>furnace repair Nashville TN</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 22:03 UTC (cycle 144)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3499,7 +3499,6 @@
           <t>https://frogair.com/</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
           <t>wecare@frogair.com</t>
@@ -3529,6 +3528,122 @@
         </is>
       </c>
       <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Rainstone Roofing Company</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>roofsoveryourhead.com</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://roofsoveryourhead.com/metal-roofing-arlington/</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Roof Replacement</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>czi@info.com</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>214-393-5217</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Arlington TX</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>100</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Arlington TX</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Kingfisher Roofing</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>kingfisher-roofing.com</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://kingfisher-roofing.com/metal-roofing/arlington/</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>info@kingfisher-roofing.com</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>(512)-831-7228</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Arlington TX</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>96</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Arlington TX</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 22:08 UTC (cycle 147)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3614,7 +3614,6 @@
           <t>https://kingfisher-roofing.com/metal-roofing/arlington/</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>info@kingfisher-roofing.com</t>
@@ -3644,6 +3643,66 @@
         </is>
       </c>
       <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>3:16 Roofing and Construction</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>316roofingtx.com</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://www.316roofingtx.com/frisco-roofing</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Construction Reviewed</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>example@mysite.com</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>817-402-7663</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Frisco TX</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>90</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>roofing contractor Frisco TX</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 22:09 UTC (cycle 148)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3708,6 +3708,66 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Custom Cooling &amp; Heating - Lincoln, NE &amp; Surrounding Areas</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>customcooling.net</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://www.customcooling.net/</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Brad Ohlmann</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>info@customcooling.net</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>402-489-9227</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Lincoln NE</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>90</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>heating and cooling company Lincoln NE</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 22:12 UTC (cycle 150)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3768,6 +3768,66 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>AC Repair Sterling Heights Hills, MI | Moreno Mechanical</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>morenomechanical.com</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://morenomechanical.com/ac-repair-sterling-heights-mi</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Read More</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>jjmoreno21@hotmail.com</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>(248) 342-9571</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>88</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>air conditioning repair Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 22:13 UTC (cycle 151)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3828,6 +3828,66 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Deck Builder Asheville NC</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>deckbuilderashevillenc.com</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://deckbuilderashevillenc.com/services/roofing/</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Asheville Area</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>deckbuilderashevillenc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>(828) 808-0838</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Asheville NC</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>90</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>roofing contractor Asheville NC</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 22:22 UTC (cycle 157)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3888,6 +3888,66 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>AC Repair &amp; Replacements | Little Rock, AR | AC Pros of Arkansas</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>acprosofarkansas.com</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://www.acprosofarkansas.com/air-conditioning-repair</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Air Conditioning</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>acprosofarkansas@gmail.com</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>501-747-9270</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Little Rock AR</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>100</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>air conditioning repair Little Rock AR</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 22:41 UTC (cycle 170)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3948,6 +3948,66 @@
         </is>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Amish Roofers</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>amish-roofers.com</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://www.amish-roofers.com/</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Free Roof</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>sales@amish-roofers.com</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>812-650-2475</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Bloomington IN</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>90</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>roofer Bloomington IN</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 22:44 UTC (cycle 172)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4008,6 +4008,66 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Roofing &amp; Siding</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>roofingandsidingofcapecod.com</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://roofingandsidingofcapecod.com/locations/boston-metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Clients Discover</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>customersupport@roofingandsidingofcapecod.com</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>(508) 360-2749</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Boston MA</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>100</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Boston MA</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 22:52 UTC (cycle 178)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4068,6 +4068,62 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>The Trade Source Mechanical LLC</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>thetradesourcemechanical.com</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://thetradesourcemechanical.com/</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>thetradesource@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>(208) 412-6713</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Boise ID</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>100</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>HVAC contractor Boise ID</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 23:00 UTC (cycle 183)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L63"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4089,7 +4089,6 @@
           <t>https://thetradesourcemechanical.com/</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
           <t>thetradesource@yahoo.com</t>
@@ -4119,6 +4118,66 @@
         </is>
       </c>
       <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Eiber Lake Plumbers</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>lakewoodcoemergencyplumbing.com</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://lakewoodcoemergencyplumbing.com/service-areas/pueblo-co/</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Eiber Lake</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>permits@prbd.com</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>(720) 704-4433</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Pueblo CO</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>90</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>emergency plumber Pueblo CO</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 23:04 UTC (cycle 186)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4183,6 +4183,62 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>AC Repair &amp; Installation Jonesboro, AR</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>evergreenhvacpro.com</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://evergreenhvacpro.com/ac-repair-installation-jonesboro-ar/</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>info@evergreenhvacpro.com</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>(833) 435-3815</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Jonesboro AR</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>90</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>AC installation Jonesboro AR</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 23:07 UTC (cycle 188)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4204,7 +4204,6 @@
           <t>https://evergreenhvacpro.com/ac-repair-installation-jonesboro-ar/</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
           <t>info@evergreenhvacpro.com</t>
@@ -4234,6 +4233,62 @@
         </is>
       </c>
       <c r="L65" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Major League Comfort Systems Heating and Air</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>majorleagueac.com</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://www.majorleagueac.com/escondido-ca-heating-air-conditioning-contractor/</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>mljshute@gmail.com</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>760-945-0975</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Escondido CA</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>100</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>heating and cooling company Escondido CA</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 23:10 UTC (cycle 190)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4259,7 +4259,6 @@
           <t>https://www.majorleagueac.com/escondido-ca-heating-air-conditioning-contractor/</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
           <t>mljshute@gmail.com</t>
@@ -4289,6 +4288,122 @@
         </is>
       </c>
       <c r="L66" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>RooterMan - Topeka</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>rootermanneks.com</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://rootermanneks.com/services/sewer-line-repair/</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>klapointe@letezsolutionsdoit.com</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>(833) 470 4376</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Topeka KS</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>100</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>sewer repair Topeka KS</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>First Roofing</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>firstroofingllc.com</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://firstroofingllc.com/fontana-ca/</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Why Fontana</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>info@firstroofingllc.com</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>(909) 323-3368</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Fontana CA</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>100</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>roofer Fontana CA</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 23:11 UTC (cycle 191)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4314,7 +4314,6 @@
           <t>https://rootermanneks.com/services/sewer-line-repair/</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
           <t>klapointe@letezsolutionsdoit.com</t>
@@ -4404,6 +4403,62 @@
         </is>
       </c>
       <c r="L68" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Standard Roofing &amp; Restoration</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>standardroofingandrestoration.com</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://standardroofingandrestoration.com/wisconsin/racine/</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>jaketheroofer@gmail.com</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>(262) 212-5853</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Racine WI</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>88</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>residential roofing company Racine WI</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 23:20 UTC (cycle 197)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4429,7 +4429,6 @@
           <t>https://standardroofingandrestoration.com/wisconsin/racine/</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
           <t>jaketheroofer@gmail.com</t>
@@ -4459,6 +4458,66 @@
         </is>
       </c>
       <c r="L69" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Performance Plumbing and Drain</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>performanceplumbing.pro</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://performanceplumbing.pro/</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Services Locations</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>info@performanceplumbing.pro</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>(406) 550-6331</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Bozeman MT</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>100</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>plumbing company Bozeman MT</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-20 23:22 UTC (cycle 198)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L70"/>
+  <dimension ref="A1:L71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4523,6 +4523,66 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Columbus Metal Roofing -</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>columbusmetalroofingoh.com</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://columbusmetalroofingoh.com/</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Surrounding Areas</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>info@columbusmetalroofingoh.com</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>740-240-0761</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Columbus OH</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>100</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Columbus OH</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 23:24 UTC (cycle 200)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4583,6 +4583,122 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Siders Roofing, LLC</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>sidersroofingia.com</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://www.sidersroofingia.com/ankeny-ia/</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Des Moines</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>sidersroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>(515) 250-7053</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Ankeny IA</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>90</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>roof replacement Ankeny IA</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Drain Cleaning Services in Yonkers, NY</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>yonkers-ny.correctplumbinganddrain.com</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://yonkers-ny.correctplumbinganddrain.com/</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>artor@correctplumbinganddrain.com</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>(917) 423-6348</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Yonkers NY</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>90</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>drain cleaning service Yonkers NY</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-20 23:35 UTC (cycle 207)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-20.xlsx
+++ b/output/leads_2026-09-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L73"/>
+  <dimension ref="A1:L74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4664,7 +4664,6 @@
           <t>https://yonkers-ny.correctplumbinganddrain.com/</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
           <t>artor@correctplumbinganddrain.com</t>
@@ -4694,6 +4693,66 @@
         </is>
       </c>
       <c r="L73" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Toms River Roofer | Roofers in Toms River</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>lgcroofing.com</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://lgcroofing.com/roof-repairs-toms-river/</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Toms River</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>lgcroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>(609) 712-8157</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Toms River NJ</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>100</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>roof repair company Toms River NJ</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>

</xml_diff>